<commit_message>
paperboy - start rta-timing version
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57ACE6D2-6290-4FD2-A364-6874305F5306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03D50A3-7AB6-4D36-AACC-314AE57E98AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46980" yWindow="3840" windowWidth="10245" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43560" yWindow="3915" windowWidth="13440" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="418">
   <si>
     <t>Place</t>
   </si>
@@ -1224,6 +1224,72 @@
   </si>
   <si>
     <t>Tuesday</t>
+  </si>
+  <si>
+    <t>crash</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>1st block</t>
+  </si>
+  <si>
+    <t>bulbs</t>
+  </si>
+  <si>
+    <t>2nd block</t>
+  </si>
+  <si>
+    <t>a 3rd but too late</t>
+  </si>
+  <si>
+    <t>0 bulbs</t>
+  </si>
+  <si>
+    <t>jack hammer guy</t>
+  </si>
+  <si>
+    <t>enemy</t>
+  </si>
+  <si>
+    <t>RNG</t>
+  </si>
+  <si>
+    <t>at</t>
+  </si>
+  <si>
+    <t>lawn mower</t>
+  </si>
+  <si>
+    <t>1st bulb</t>
+  </si>
+  <si>
+    <t>1st 2</t>
+  </si>
+  <si>
+    <t>1st 3</t>
+  </si>
+  <si>
+    <t>dog!!!!!!</t>
+  </si>
+  <si>
+    <t>probable frame savings (could be more)</t>
+  </si>
+  <si>
+    <t>53 when passing the last bulb = doggo</t>
   </si>
 </sst>
 </file>
@@ -1233,12 +1299,26 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="39" x14ac:knownFonts="1">
+  <fonts count="41" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1721,95 +1801,97 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1830,35 +1912,37 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="14" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" xfId="6" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2179,16 +2263,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F185"/>
+  <dimension ref="A1:I185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="8.75" customWidth="1"/>
     <col min="4" max="4" width="6.625" customWidth="1"/>
     <col min="5" max="5" width="17.625" style="51" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2202,8 +2287,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="54" t="s">
         <v>391</v>
       </c>
       <c r="B2" s="2">
@@ -2216,39 +2301,62 @@
         <f t="shared" ref="D2:D18" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="F2" t="s">
+        <v>402</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="55" t="s">
         <v>392</v>
       </c>
-      <c r="B3" s="64">
+      <c r="B3" s="56">
         <v>17</v>
       </c>
-      <c r="C3" s="64">
+      <c r="C3" s="56">
         <v>18</v>
       </c>
-      <c r="D3" s="65">
+      <c r="D3" s="57">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="62" t="s">
+      <c r="F3" t="s">
+        <v>404</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="54" t="s">
         <v>393</v>
       </c>
       <c r="B4" s="2">
-        <v>618</v>
+        <v>1609</v>
       </c>
       <c r="C4" s="2">
         <v>619</v>
       </c>
       <c r="D4" s="3">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="62" t="s">
+        <v>-990</v>
+      </c>
+      <c r="E4" s="2">
+        <v>618</v>
+      </c>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="54" t="s">
         <v>394</v>
       </c>
       <c r="B5" s="2">
@@ -2261,127 +2369,271 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
-        <v>392</v>
-      </c>
-      <c r="B6" s="2">
-        <v>5726</v>
-      </c>
-      <c r="C6" s="2">
-        <v>5391</v>
-      </c>
-      <c r="D6" s="3">
-        <f t="shared" si="0"/>
-        <v>-335</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="62" t="s">
+      <c r="E5" s="2">
+        <v>886</v>
+      </c>
+      <c r="F5" s="58"/>
+      <c r="G5" s="61" t="s">
+        <v>408</v>
+      </c>
+      <c r="H5" t="s">
+        <v>409</v>
+      </c>
+      <c r="I5" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="59" t="s">
+        <v>396</v>
+      </c>
+      <c r="B6" s="56">
+        <v>6087</v>
+      </c>
+      <c r="C6" s="56">
+        <v>5150</v>
+      </c>
+      <c r="D6" s="57">
+        <f t="shared" si="0"/>
+        <v>-937</v>
+      </c>
+      <c r="E6" s="56">
+        <v>5149</v>
+      </c>
+      <c r="F6" s="61" t="s">
+        <v>406</v>
+      </c>
+      <c r="G6" s="61" t="s">
+        <v>407</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>5939</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="54" t="s">
         <v>395</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="50"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="50"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="50"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="50"/>
+      <c r="B7" s="2">
+        <v>7202</v>
+      </c>
+      <c r="C7" s="2">
+        <v>6265</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>-937</v>
+      </c>
+      <c r="E7" s="2">
+        <v>6264</v>
+      </c>
+      <c r="F7" s="61" t="s">
+        <v>412</v>
+      </c>
+      <c r="G7" s="61" t="s">
+        <v>411</v>
+      </c>
+      <c r="H7">
+        <v>52</v>
+      </c>
+      <c r="I7">
+        <v>5939</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="59" t="s">
+        <v>396</v>
+      </c>
+      <c r="B8" s="60">
+        <v>11686</v>
+      </c>
+      <c r="C8" s="60">
+        <v>10824</v>
+      </c>
+      <c r="D8" s="57">
+        <f t="shared" si="0"/>
+        <v>-862</v>
+      </c>
+      <c r="E8" s="60">
+        <v>10822</v>
+      </c>
+      <c r="F8" s="61" t="s">
+        <v>413</v>
+      </c>
+      <c r="G8" s="61" t="s">
+        <v>407</v>
+      </c>
+      <c r="H8">
+        <v>17</v>
+      </c>
+      <c r="I8">
+        <v>5939</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="58" t="s">
+        <v>397</v>
+      </c>
+      <c r="B9" s="7">
+        <v>12801</v>
+      </c>
+      <c r="C9" s="7">
+        <v>11939</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>-862</v>
+      </c>
+      <c r="E9" s="7">
+        <v>11937</v>
+      </c>
+      <c r="F9" s="61" t="s">
+        <v>414</v>
+      </c>
+      <c r="G9" s="61" t="s">
+        <v>415</v>
+      </c>
+      <c r="H9">
+        <v>47</v>
+      </c>
+      <c r="I9">
+        <v>5939</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="59" t="s">
+        <v>396</v>
+      </c>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60">
+        <v>16489</v>
+      </c>
+      <c r="D10" s="57" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E10" s="58">
+        <f>(D6-D4)*7</f>
+        <v>371</v>
+      </c>
+      <c r="F10" s="61" t="s">
+        <v>416</v>
+      </c>
+      <c r="G10" s="58"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="58" t="s">
+        <v>398</v>
+      </c>
       <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
+      <c r="C11" s="7">
+        <v>17604</v>
+      </c>
       <c r="D11" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="50"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="50"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="59" t="s">
+        <v>396</v>
+      </c>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60">
+        <v>22211</v>
+      </c>
+      <c r="D12" s="57" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E12" s="58"/>
+      <c r="F12" s="61" t="s">
+        <v>417</v>
+      </c>
+      <c r="G12" s="58"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="58" t="s">
+        <v>399</v>
+      </c>
       <c r="B13" s="7"/>
-      <c r="C13" s="37"/>
+      <c r="C13" s="37">
+        <v>23326</v>
+      </c>
       <c r="D13" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="50"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="50"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="59" t="s">
+        <v>396</v>
+      </c>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60">
+        <v>27992</v>
+      </c>
+      <c r="D14" s="57" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="58" t="s">
+        <v>400</v>
+      </c>
       <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="C15" s="7">
+        <v>29107</v>
+      </c>
       <c r="D15" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="50"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="3" t="str">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="59" t="s">
+        <v>396</v>
+      </c>
+      <c r="B16" s="60"/>
+      <c r="C16" s="60">
+        <v>33801</v>
+      </c>
+      <c r="D16" s="57" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="50"/>
+      <c r="A17" s="58" t="s">
+        <v>401</v>
+      </c>
       <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
+      <c r="C17" s="7">
+        <v>34916</v>
+      </c>
       <c r="D17" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="50"/>
+      <c r="A18" s="58" t="s">
+        <v>26</v>
+      </c>
       <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
+      <c r="C18" s="7">
+        <v>40853</v>
+      </c>
       <c r="D18" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
@@ -18365,7 +18617,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="35" type="noConversion"/>
+  <phoneticPr fontId="37" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -18395,10 +18647,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="54" t="s">
+      <c r="K1" s="62" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="55"/>
+      <c r="L1" s="63"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20250,13 +20502,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="56" t="s">
+      <c r="H53" s="64" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="57"/>
-      <c r="J53" s="57"/>
-      <c r="K53" s="57"/>
-      <c r="L53" s="58"/>
+      <c r="I53" s="65"/>
+      <c r="J53" s="65"/>
+      <c r="K53" s="65"/>
+      <c r="L53" s="66"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20278,11 +20530,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="59"/>
-      <c r="I54" s="60"/>
-      <c r="J54" s="60"/>
-      <c r="K54" s="60"/>
-      <c r="L54" s="61"/>
+      <c r="H54" s="67"/>
+      <c r="I54" s="68"/>
+      <c r="J54" s="68"/>
+      <c r="K54" s="68"/>
+      <c r="L54" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
paperboy - rta v1 done, can definitely end input sooner, and maybe lag management can improve some days, entertaining things still need to be added as well
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03D50A3-7AB6-4D36-AACC-314AE57E98AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5FA885E-F4CA-4DC3-BE4C-D8D91653E3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43560" yWindow="3915" windowWidth="13440" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2507,13 +2507,15 @@
       <c r="A10" s="59" t="s">
         <v>396</v>
       </c>
-      <c r="B10" s="60"/>
+      <c r="B10" s="60">
+        <v>17290</v>
+      </c>
       <c r="C10" s="60">
         <v>16489</v>
       </c>
-      <c r="D10" s="57" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D10" s="57">
+        <f t="shared" si="0"/>
+        <v>-801</v>
       </c>
       <c r="E10" s="58">
         <f>(D6-D4)*7</f>
@@ -2528,13 +2530,15 @@
       <c r="A11" s="58" t="s">
         <v>398</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="7">
+        <v>18405</v>
+      </c>
       <c r="C11" s="7">
         <v>17604</v>
       </c>
-      <c r="D11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>-801</v>
       </c>
       <c r="E11" s="58"/>
       <c r="F11" s="58"/>
@@ -2544,13 +2548,15 @@
       <c r="A12" s="59" t="s">
         <v>396</v>
       </c>
-      <c r="B12" s="60"/>
+      <c r="B12" s="60">
+        <v>22912</v>
+      </c>
       <c r="C12" s="60">
         <v>22211</v>
       </c>
-      <c r="D12" s="57" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D12" s="57">
+        <f t="shared" si="0"/>
+        <v>-701</v>
       </c>
       <c r="E12" s="58"/>
       <c r="F12" s="61" t="s">
@@ -2562,13 +2568,15 @@
       <c r="A13" s="58" t="s">
         <v>399</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="7">
+        <v>24027</v>
+      </c>
       <c r="C13" s="37">
         <v>23326</v>
       </c>
-      <c r="D13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>-701</v>
       </c>
       <c r="E13" s="58"/>
       <c r="F13" s="58"/>
@@ -2578,65 +2586,75 @@
       <c r="A14" s="59" t="s">
         <v>396</v>
       </c>
-      <c r="B14" s="60"/>
+      <c r="B14" s="60">
+        <v>28563</v>
+      </c>
       <c r="C14" s="60">
         <v>27992</v>
       </c>
-      <c r="D14" s="57" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D14" s="57">
+        <f t="shared" si="0"/>
+        <v>-571</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="58" t="s">
         <v>400</v>
       </c>
-      <c r="B15" s="7"/>
+      <c r="B15" s="7">
+        <v>29678</v>
+      </c>
       <c r="C15" s="7">
         <v>29107</v>
       </c>
-      <c r="D15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>-571</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="59" t="s">
         <v>396</v>
       </c>
-      <c r="B16" s="60"/>
+      <c r="B16" s="60">
+        <v>34302</v>
+      </c>
       <c r="C16" s="60">
         <v>33801</v>
       </c>
-      <c r="D16" s="57" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D16" s="57">
+        <f t="shared" si="0"/>
+        <v>-501</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="58" t="s">
         <v>401</v>
       </c>
-      <c r="B17" s="7"/>
+      <c r="B17" s="7">
+        <v>35417</v>
+      </c>
       <c r="C17" s="7">
         <v>34916</v>
       </c>
-      <c r="D17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D17" s="3">
+        <f t="shared" si="0"/>
+        <v>-501</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="7"/>
+      <c r="B18" s="7">
+        <v>39864</v>
+      </c>
       <c r="C18" s="7">
         <v>40853</v>
       </c>
-      <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>989</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
paper boy rta timing v2 - 257 faster (96 actual, rest is ending input sooner)
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF37FC75-7266-4CB2-BA8D-28FD464C6A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05E52B3-BF00-40A0-BA92-6D4EEE8058F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36030" yWindow="2220" windowWidth="11190" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V2" sheetId="9" r:id="rId1"/>
     <sheet name="V1" sheetId="8" r:id="rId2"/>
+    <sheet name="Bulb Check" sheetId="10" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="74">
   <si>
     <t>Place</t>
   </si>
@@ -142,6 +143,117 @@
   </si>
   <si>
     <t>Monday (1st input frame)</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>B13</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>B12</t>
+  </si>
+  <si>
+    <t>B1-B2</t>
+  </si>
+  <si>
+    <t>B1-B3</t>
+  </si>
+  <si>
+    <t>B1-B12</t>
+  </si>
+  <si>
+    <t>B1-B13</t>
+  </si>
+  <si>
+    <t>B2-B3</t>
+  </si>
+  <si>
+    <t>B2-B12</t>
+  </si>
+  <si>
+    <t>B2-B13</t>
+  </si>
+  <si>
+    <t>B3-B12</t>
+  </si>
+  <si>
+    <t>B3-B13</t>
+  </si>
+  <si>
+    <t>B12-B13</t>
+  </si>
+  <si>
+    <t>B1-B2-B3</t>
+  </si>
+  <si>
+    <t>B1-B2-B12</t>
+  </si>
+  <si>
+    <t>B1-B2-B13</t>
+  </si>
+  <si>
+    <t>B1-B3-B12</t>
+  </si>
+  <si>
+    <t>B1-B3-B13</t>
+  </si>
+  <si>
+    <t>B1-B12-B13</t>
+  </si>
+  <si>
+    <t>B2-B3-B12</t>
+  </si>
+  <si>
+    <t>B2-B3-B13</t>
+  </si>
+  <si>
+    <t>B2-B12-B13</t>
+  </si>
+  <si>
+    <t>B3-B12-B13</t>
+  </si>
+  <si>
+    <t>B1-B2-B3-B12</t>
+  </si>
+  <si>
+    <t>B1-B2-B3-B13</t>
+  </si>
+  <si>
+    <t>B1-B2-B12-B13</t>
+  </si>
+  <si>
+    <t>B1-B3-B12-B13</t>
+  </si>
+  <si>
+    <t>B2-B3-B12-B13</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Tuesday (1st input frame)</t>
+  </si>
+  <si>
+    <t>crash (lag frame)</t>
+  </si>
+  <si>
+    <t>Block 2: 2 lag</t>
+  </si>
+  <si>
+    <t>Block 1: 3 lag</t>
   </si>
 </sst>
 </file>
@@ -151,12 +263,47 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -335,42 +482,48 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -698,6 +851,7 @@
     <col min="2" max="3" width="8.75" customWidth="1"/>
     <col min="4" max="4" width="6.625" customWidth="1"/>
     <col min="5" max="5" width="17.625" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -750,14 +904,14 @@
         <v>35</v>
       </c>
       <c r="B4" s="15">
-        <v>540</v>
+        <v>924</v>
       </c>
       <c r="C4" s="15">
         <v>980</v>
       </c>
       <c r="D4" s="16">
         <f t="shared" si="0"/>
-        <v>440</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -765,229 +919,258 @@
         <v>36</v>
       </c>
       <c r="B5" s="2">
-        <v>1422</v>
+        <v>1804</v>
       </c>
       <c r="C5" s="2">
         <v>1877</v>
       </c>
       <c r="D5" s="3">
         <f t="shared" si="0"/>
-        <v>455</v>
+        <v>73</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>8</v>
-      </c>
+      <c r="A6" s="13"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="2">
-        <v>886</v>
-      </c>
+      <c r="C6" s="2"/>
       <c r="D6" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="20"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="15"/>
+      <c r="A7" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="15">
+        <v>6013</v>
+      </c>
       <c r="C7" s="15">
-        <v>6087</v>
-      </c>
-      <c r="D7" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>6086</v>
+      </c>
+      <c r="D7" s="16">
+        <f t="shared" si="0"/>
+        <v>73</v>
       </c>
       <c r="E7" s="15"/>
       <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
+      <c r="G7" s="24"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="2"/>
+      <c r="A8" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="2">
+        <v>7397</v>
+      </c>
       <c r="C8" s="2">
-        <v>7202</v>
-      </c>
-      <c r="D8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
+        <v>7470</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>73</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="24"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="19"/>
+      <c r="A9" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="19">
+        <v>11611</v>
+      </c>
       <c r="C9" s="19">
-        <v>11686</v>
-      </c>
-      <c r="D9" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>11685</v>
+      </c>
+      <c r="D9" s="16">
+        <f t="shared" si="0"/>
+        <v>74</v>
       </c>
       <c r="E9" s="19"/>
       <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
+      <c r="G9" s="24"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="4">
+        <v>12995</v>
+      </c>
       <c r="C10" s="4">
-        <v>12801</v>
-      </c>
-      <c r="D10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>13069</v>
+      </c>
+      <c r="D10" s="3">
+        <f t="shared" si="0"/>
+        <v>74</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
+      <c r="G10" s="24"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="19"/>
+      <c r="B11" s="19">
+        <v>17212</v>
+      </c>
       <c r="C11" s="19">
-        <v>17290</v>
-      </c>
-      <c r="D11" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>17289</v>
+      </c>
+      <c r="D11" s="16">
+        <f t="shared" si="0"/>
+        <v>77</v>
       </c>
       <c r="E11" s="17"/>
       <c r="F11" s="20"/>
-      <c r="G11" s="17"/>
+      <c r="G11" s="24"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="4"/>
+      <c r="B12" s="4">
+        <v>18596</v>
+      </c>
       <c r="C12" s="4">
-        <v>18405</v>
-      </c>
-      <c r="D12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>18673</v>
+      </c>
+      <c r="D12" s="3">
+        <f t="shared" si="0"/>
+        <v>77</v>
       </c>
       <c r="E12" s="17"/>
       <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
+      <c r="G12" s="24"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="19"/>
+      <c r="B13" s="19">
+        <v>22830</v>
+      </c>
       <c r="C13" s="19">
-        <v>22912</v>
-      </c>
-      <c r="D13" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>22911</v>
+      </c>
+      <c r="D13" s="16">
+        <f t="shared" si="0"/>
+        <v>81</v>
       </c>
       <c r="E13" s="17"/>
       <c r="F13" s="20"/>
-      <c r="G13" s="17"/>
+      <c r="G13" s="24"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4"/>
+      <c r="B14" s="4">
+        <v>24214</v>
+      </c>
       <c r="C14" s="4">
-        <v>24027</v>
-      </c>
-      <c r="D14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>24295</v>
+      </c>
+      <c r="D14" s="3">
+        <f t="shared" si="0"/>
+        <v>81</v>
       </c>
       <c r="E14" s="17"/>
       <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
+      <c r="G14" s="24"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="19"/>
+      <c r="B15" s="19">
+        <v>28470</v>
+      </c>
       <c r="C15" s="19">
-        <v>28563</v>
-      </c>
-      <c r="D15" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
+        <v>28562</v>
+      </c>
+      <c r="D15" s="16">
+        <f t="shared" si="0"/>
+        <v>92</v>
+      </c>
+      <c r="G15" s="24"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="4"/>
+      <c r="B16" s="4">
+        <v>29854</v>
+      </c>
       <c r="C16" s="4">
-        <v>29678</v>
-      </c>
-      <c r="D16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>29946</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" si="0"/>
+        <v>92</v>
+      </c>
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="19"/>
+      <c r="B17" s="29">
+        <v>34205</v>
+      </c>
       <c r="C17" s="19">
-        <v>34302</v>
-      </c>
-      <c r="D17" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34301</v>
+      </c>
+      <c r="D17" s="16">
+        <f t="shared" si="0"/>
+        <v>96</v>
+      </c>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4">
-        <v>35417</v>
+        <v>35685</v>
       </c>
       <c r="D18" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="4"/>
+      <c r="B19" s="4">
+        <v>39607</v>
+      </c>
       <c r="C19" s="4">
         <v>39864</v>
       </c>
-      <c r="D19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" s="3">
+        <f t="shared" si="0"/>
+        <v>257</v>
+      </c>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -995,8 +1178,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G20" s="24"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1004,8 +1188,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G21" s="24"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1013,8 +1198,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1022,8 +1208,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G23" s="24"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1031,8 +1218,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G24" s="24"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1040,8 +1228,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G25" s="24"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1049,8 +1238,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1058,8 +1248,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G27" s="24"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -1067,8 +1258,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G28" s="24"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="B29" s="10"/>
       <c r="C29" s="4"/>
@@ -1076,8 +1268,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G29" s="24"/>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1085,8 +1278,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G30" s="24"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -1094,8 +1288,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G31" s="24"/>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1103,6 +1298,7 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="G32" s="27"/>
     </row>
     <row r="33" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
@@ -3583,4 +3779,262 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAC1BD0-BE10-4CBC-A8BB-B931744D8671}">
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
start paperboy rta timing v3 - MOnday done, same number of frames, but attempting to put in entertainment value
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05E52B3-BF00-40A0-BA92-6D4EEE8058F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9EE5C12-0150-4F1E-A83A-D70FE57580FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="V2" sheetId="9" r:id="rId1"/>
-    <sheet name="V1" sheetId="8" r:id="rId2"/>
-    <sheet name="Bulb Check" sheetId="10" r:id="rId3"/>
+    <sheet name="V3" sheetId="11" r:id="rId1"/>
+    <sheet name="V2" sheetId="9" r:id="rId2"/>
+    <sheet name="V1" sheetId="8" r:id="rId3"/>
+    <sheet name="Bulb Check" sheetId="10" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="75">
   <si>
     <t>Place</t>
   </si>
@@ -254,6 +255,9 @@
   </si>
   <si>
     <t>Block 1: 3 lag</t>
+  </si>
+  <si>
+    <t>rta v3</t>
   </si>
 </sst>
 </file>
@@ -843,6 +847,1410 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FBDE017-57E1-41A6-9366-1949A55961DE}">
+  <dimension ref="A1:G185"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.75" customWidth="1"/>
+    <col min="4" max="4" width="6.625" customWidth="1"/>
+    <col min="5" max="5" width="17.625" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3">
+        <f t="shared" ref="D2:D65" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="15">
+        <v>281</v>
+      </c>
+      <c r="C3" s="15">
+        <v>281</v>
+      </c>
+      <c r="D3" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="15">
+        <v>924</v>
+      </c>
+      <c r="C4" s="15">
+        <v>924</v>
+      </c>
+      <c r="D4" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1804</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1804</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="15">
+        <v>6013</v>
+      </c>
+      <c r="C6" s="15">
+        <v>6013</v>
+      </c>
+      <c r="D6" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="15"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="24"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2">
+        <v>7397</v>
+      </c>
+      <c r="D7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E7" s="28"/>
+      <c r="F7" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="24"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19">
+        <v>11611</v>
+      </c>
+      <c r="D8" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="24"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4">
+        <v>12995</v>
+      </c>
+      <c r="D9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="24"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19">
+        <v>17212</v>
+      </c>
+      <c r="D10" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E10" s="17"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="24"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4">
+        <v>18596</v>
+      </c>
+      <c r="D11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="24"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19">
+        <v>22830</v>
+      </c>
+      <c r="D12" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E12" s="17"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="24"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4">
+        <v>24214</v>
+      </c>
+      <c r="D13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19">
+        <v>28470</v>
+      </c>
+      <c r="D14" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G14" s="24"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4">
+        <v>29854</v>
+      </c>
+      <c r="D15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G15" s="24"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29">
+        <v>34205</v>
+      </c>
+      <c r="D16" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4">
+        <v>39607</v>
+      </c>
+      <c r="D18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="9"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G20" s="24"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G21" s="24"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G23" s="24"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G24" s="24"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G25" s="24"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="9"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="9"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G27" s="24"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="9"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G28" s="24"/>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G29" s="24"/>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G30" s="24"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G31" s="27"/>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="9"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="9"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="9"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="9"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="9"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="9"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="9"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="9"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="9"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="9"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="9"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="9"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="9"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="9"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="9"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="9"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="9"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="9"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="9"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="9"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="9"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="9"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="9"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="9"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="9"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="9"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="9"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="9"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F64" s="4"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="9"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F65" s="4"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="9"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="3" t="str">
+        <f t="shared" ref="D66:D101" si="1">IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="9"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="9"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="F68" s="4"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="9"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="F69" s="4"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="9"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="9"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="9"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="9"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="9"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="9"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="9"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="9"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="9"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="9"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="9"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="9"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="9"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E82" s="12"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="9"/>
+      <c r="B83" s="12"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="9"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="9"/>
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="9"/>
+      <c r="B86" s="4"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E86" s="4"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="9"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="9"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="9"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="9"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="9"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="9"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="9"/>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="9"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="9"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="9"/>
+      <c r="B96" s="6"/>
+      <c r="C96" s="6"/>
+      <c r="D96" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="9"/>
+      <c r="B97" s="4"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="9"/>
+      <c r="B98" s="4"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="9"/>
+      <c r="B99" s="4"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E99" s="4"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="9"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="9"/>
+      <c r="B101" s="4"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B102" s="4"/>
+      <c r="C102" s="4"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B103" s="4"/>
+      <c r="C103" s="4"/>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B105" s="4"/>
+      <c r="C105" s="4"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="3"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B107" s="4"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="3"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B108" s="4"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="3"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B109" s="4"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="3"/>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B110" s="4"/>
+      <c r="C110" s="4"/>
+      <c r="D110" s="3"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B111" s="4"/>
+      <c r="C111" s="4"/>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B112" s="4"/>
+      <c r="C112" s="4"/>
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B113" s="4"/>
+      <c r="C113" s="4"/>
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B114" s="4"/>
+      <c r="C114" s="4"/>
+    </row>
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B115" s="4"/>
+      <c r="C115" s="4"/>
+    </row>
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B116" s="4"/>
+      <c r="C116" s="4"/>
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B117" s="4"/>
+      <c r="C117" s="4"/>
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B118" s="4"/>
+      <c r="C118" s="4"/>
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B119" s="4"/>
+      <c r="C119" s="4"/>
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B120" s="4"/>
+      <c r="C120" s="4"/>
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B121" s="4"/>
+      <c r="C121" s="4"/>
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B122" s="4"/>
+      <c r="C122" s="4"/>
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B123" s="4"/>
+      <c r="C123" s="4"/>
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B124" s="4"/>
+      <c r="C124" s="4"/>
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B125" s="4"/>
+      <c r="C125" s="4"/>
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B126" s="4"/>
+      <c r="C126" s="4"/>
+    </row>
+    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B127" s="4"/>
+      <c r="C127" s="4"/>
+    </row>
+    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B128" s="4"/>
+      <c r="C128" s="4"/>
+    </row>
+    <row r="129" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B129" s="4"/>
+      <c r="C129" s="4"/>
+    </row>
+    <row r="130" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B130" s="4"/>
+      <c r="C130" s="4"/>
+    </row>
+    <row r="131" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B131" s="4"/>
+      <c r="C131" s="4"/>
+    </row>
+    <row r="132" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B132" s="4"/>
+      <c r="C132" s="4"/>
+    </row>
+    <row r="133" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B133" s="4"/>
+      <c r="C133" s="4"/>
+    </row>
+    <row r="134" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B134" s="4"/>
+      <c r="C134" s="4"/>
+    </row>
+    <row r="135" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B135" s="4"/>
+      <c r="C135" s="4"/>
+    </row>
+    <row r="136" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B136" s="4"/>
+      <c r="C136" s="4"/>
+    </row>
+    <row r="137" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B137" s="4"/>
+      <c r="C137" s="4"/>
+    </row>
+    <row r="138" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B138" s="4"/>
+      <c r="C138" s="4"/>
+    </row>
+    <row r="139" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B139" s="4"/>
+      <c r="C139" s="4"/>
+    </row>
+    <row r="140" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B140" s="4"/>
+      <c r="C140" s="4"/>
+    </row>
+    <row r="141" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B141" s="4"/>
+      <c r="C141" s="4"/>
+    </row>
+    <row r="142" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B142" s="4"/>
+      <c r="C142" s="4"/>
+    </row>
+    <row r="143" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B143" s="4"/>
+      <c r="C143" s="4"/>
+    </row>
+    <row r="144" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B144" s="4"/>
+      <c r="C144" s="4"/>
+    </row>
+    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B145" s="4"/>
+      <c r="C145" s="4"/>
+    </row>
+    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B146" s="4"/>
+      <c r="C146" s="4"/>
+    </row>
+    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B147" s="4"/>
+      <c r="C147" s="4"/>
+    </row>
+    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B148" s="4"/>
+      <c r="C148" s="4"/>
+    </row>
+    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B149" s="4"/>
+      <c r="C149" s="4"/>
+    </row>
+    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B150" s="4"/>
+      <c r="C150" s="4"/>
+    </row>
+    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B151" s="4"/>
+      <c r="C151" s="4"/>
+    </row>
+    <row r="152" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B152" s="4"/>
+      <c r="C152" s="4"/>
+    </row>
+    <row r="153" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B153" s="4"/>
+      <c r="C153" s="4"/>
+    </row>
+    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B154" s="4"/>
+      <c r="C154" s="4"/>
+    </row>
+    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B155" s="4"/>
+      <c r="C155" s="4"/>
+    </row>
+    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B156" s="4"/>
+      <c r="C156" s="4"/>
+    </row>
+    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B157" s="4"/>
+      <c r="C157" s="4"/>
+    </row>
+    <row r="158" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B158" s="4"/>
+      <c r="C158" s="4"/>
+    </row>
+    <row r="159" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B159" s="4"/>
+      <c r="C159" s="4"/>
+    </row>
+    <row r="160" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B160" s="4"/>
+      <c r="C160" s="4"/>
+    </row>
+    <row r="161" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B161" s="4"/>
+      <c r="C161" s="4"/>
+    </row>
+    <row r="162" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B162" s="4"/>
+      <c r="C162" s="4"/>
+    </row>
+    <row r="163" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B163" s="4"/>
+      <c r="C163" s="4"/>
+    </row>
+    <row r="164" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B164" s="4"/>
+      <c r="C164" s="4"/>
+    </row>
+    <row r="165" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B165" s="4"/>
+      <c r="C165" s="4"/>
+    </row>
+    <row r="166" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B166" s="4"/>
+      <c r="C166" s="4"/>
+    </row>
+    <row r="167" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B167" s="4"/>
+      <c r="C167" s="4"/>
+    </row>
+    <row r="168" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B168" s="4"/>
+      <c r="C168" s="4"/>
+    </row>
+    <row r="169" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B169" s="4"/>
+      <c r="C169" s="4"/>
+    </row>
+    <row r="170" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B170" s="4"/>
+      <c r="C170" s="4"/>
+    </row>
+    <row r="171" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B171" s="4"/>
+      <c r="C171" s="4"/>
+    </row>
+    <row r="172" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B172" s="4"/>
+      <c r="C172" s="4"/>
+    </row>
+    <row r="173" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B173" s="4"/>
+      <c r="C173" s="4"/>
+    </row>
+    <row r="174" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B174" s="4"/>
+      <c r="C174" s="4"/>
+    </row>
+    <row r="175" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B175" s="4"/>
+      <c r="C175" s="4"/>
+    </row>
+    <row r="176" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B176" s="4"/>
+      <c r="C176" s="4"/>
+    </row>
+    <row r="177" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B177" s="4"/>
+      <c r="C177" s="4"/>
+    </row>
+    <row r="178" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B178" s="4"/>
+      <c r="C178" s="4"/>
+    </row>
+    <row r="179" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B179" s="4"/>
+      <c r="C179" s="4"/>
+    </row>
+    <row r="180" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B180" s="4"/>
+      <c r="C180" s="4"/>
+    </row>
+    <row r="181" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B181" s="4"/>
+      <c r="C181" s="4"/>
+    </row>
+    <row r="182" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B182" s="4"/>
+      <c r="C182" s="4"/>
+    </row>
+    <row r="183" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B183" s="4"/>
+      <c r="C183" s="4"/>
+    </row>
+    <row r="184" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B184" s="4"/>
+      <c r="C184" s="4"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="4"/>
+      <c r="C185" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1983864C-ED7D-4E0B-969E-AE843FEB855D}">
   <dimension ref="A1:G186"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2284,7 +3692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
   <dimension ref="A1:I185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3781,7 +5189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAC1BD0-BE10-4CBC-A8BB-B931744D8671}">
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
paperboy v3 - Wednesday done
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9EE5C12-0150-4F1E-A83A-D70FE57580FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4404BB2A-110A-4415-8620-B4529B822070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -958,13 +958,15 @@
       <c r="A7" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" s="2">
+        <v>7397</v>
+      </c>
       <c r="C7" s="2">
         <v>7397</v>
       </c>
-      <c r="D7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="E7" s="28"/>
       <c r="F7" s="27" t="s">
@@ -976,13 +978,15 @@
       <c r="A8" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="19"/>
+      <c r="B8" s="19">
+        <v>11611</v>
+      </c>
       <c r="C8" s="19">
         <v>11611</v>
       </c>
-      <c r="D8" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D8" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
@@ -992,13 +996,15 @@
       <c r="A9" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="4">
+        <v>12995</v>
+      </c>
       <c r="C9" s="4">
         <v>12995</v>
       </c>
-      <c r="D9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="20"/>
@@ -1008,13 +1014,15 @@
       <c r="A10" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="19"/>
+      <c r="B10" s="19">
+        <v>17212</v>
+      </c>
       <c r="C10" s="19">
         <v>17212</v>
       </c>
-      <c r="D10" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D10" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="E10" s="17"/>
       <c r="F10" s="20"/>
@@ -1024,13 +1032,15 @@
       <c r="A11" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="4">
+        <v>18596</v>
+      </c>
       <c r="C11" s="4">
         <v>18596</v>
       </c>
-      <c r="D11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>

</xml_diff>

<commit_message>
paperboy v3 - thursday done, 2 lag frames saved
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4404BB2A-110A-4415-8620-B4529B822070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112B5C8E-17AC-4577-BDBC-99D6E43930DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1050,13 +1050,15 @@
       <c r="A12" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="19"/>
+      <c r="B12" s="19">
+        <v>22828</v>
+      </c>
       <c r="C12" s="19">
         <v>22830</v>
       </c>
-      <c r="D12" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D12" s="16">
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="E12" s="17"/>
       <c r="F12" s="20"/>
@@ -1066,13 +1068,15 @@
       <c r="A13" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="4"/>
+      <c r="B13" s="4">
+        <v>24212</v>
+      </c>
       <c r="C13" s="4">
         <v>24214</v>
       </c>
-      <c r="D13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="E13" s="17"/>
       <c r="F13" s="17"/>

</xml_diff>

<commit_message>
paperboy v3 - friday done - 7 frames ahead
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112B5C8E-17AC-4577-BDBC-99D6E43930DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A77813-733C-4F36-B0FE-020DF47AC23D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49605" yWindow="4005" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V3" sheetId="11" r:id="rId1"/>
@@ -1086,13 +1086,15 @@
       <c r="A14" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="19"/>
+      <c r="B14" s="19">
+        <v>28463</v>
+      </c>
       <c r="C14" s="19">
         <v>28470</v>
       </c>
-      <c r="D14" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D14" s="16">
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="G14" s="24"/>
     </row>
@@ -1100,13 +1102,15 @@
       <c r="A15" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="4"/>
+      <c r="B15" s="4">
+        <v>29847</v>
+      </c>
       <c r="C15" s="4">
         <v>29854</v>
       </c>
-      <c r="D15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="G15" s="24"/>
     </row>

</xml_diff>

<commit_message>
paperboy v3 - friday - 1 frame saved using U+D, this looks useful in general to reduce lag
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A77813-733C-4F36-B0FE-020DF47AC23D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0757F839-AB67-42AE-8A54-960A6AF173E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49605" yWindow="4005" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1087,14 +1087,14 @@
         <v>10</v>
       </c>
       <c r="B14" s="19">
-        <v>28463</v>
+        <v>28462</v>
       </c>
       <c r="C14" s="19">
         <v>28470</v>
       </c>
       <c r="D14" s="16">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G14" s="24"/>
     </row>
@@ -1103,14 +1103,14 @@
         <v>14</v>
       </c>
       <c r="B15" s="4">
-        <v>29847</v>
+        <v>29846</v>
       </c>
       <c r="C15" s="4">
         <v>29854</v>
       </c>
       <c r="D15" s="3">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G15" s="24"/>
     </row>

</xml_diff>

<commit_message>
paperboy v3 - saturday done, 14 frames ahead
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0757F839-AB67-42AE-8A54-960A6AF173E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012FC0F0-1AA3-4C86-BE3E-33D94406361E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49605" yWindow="4005" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V3" sheetId="11" r:id="rId1"/>
@@ -1118,13 +1118,15 @@
       <c r="A16" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="29"/>
+      <c r="B16" s="29">
+        <v>34191</v>
+      </c>
       <c r="C16" s="29">
         <v>34205</v>
       </c>
-      <c r="D16" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D16" s="16">
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="G16" s="24"/>
     </row>

</xml_diff>

<commit_message>
paperboy rta v3 done, 39967, and the actual ending.  v1 & 2 end input early but that does not work for rta timing
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012FC0F0-1AA3-4C86-BE3E-33D94406361E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DF878D-E661-44C6-ACB2-3F005DFDBEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V3" sheetId="11" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="75">
   <si>
     <t>Place</t>
   </si>
@@ -267,12 +267,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -486,22 +493,23 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -511,23 +519,23 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -848,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FBDE017-57E1-41A6-9366-1949A55961DE}">
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
@@ -884,7 +892,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D65" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D67" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>0</v>
       </c>
     </row>
@@ -1143,36 +1151,48 @@
       <c r="G17" s="24"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="17"/>
+      <c r="B18" s="4">
+        <v>9516</v>
+      </c>
+      <c r="C18" s="4">
+        <v>9535</v>
+      </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4">
+        <v>9560</v>
+      </c>
+      <c r="C19" s="4">
+        <v>9579</v>
+      </c>
+      <c r="D19" s="3">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4">
+      <c r="B20" s="4">
+        <v>39524</v>
+      </c>
+      <c r="C20" s="4">
         <v>39607</v>
       </c>
-      <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G18" s="24"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G19" s="24"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D20" s="3">
+        <f t="shared" si="0"/>
+        <v>83</v>
       </c>
       <c r="G20" s="24"/>
     </row>
@@ -1248,7 +1268,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
-      <c r="B28" s="10"/>
+      <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1256,7 +1276,7 @@
       </c>
       <c r="G28" s="24"/>
     </row>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1266,9 +1286,9 @@
       </c>
       <c r="G29" s="24"/>
     </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
-      <c r="B30" s="4"/>
+      <c r="B30" s="10"/>
       <c r="C30" s="4"/>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1284,7 +1304,7 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="G31" s="27"/>
+      <c r="G31" s="24"/>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
@@ -1294,8 +1314,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G32" s="24"/>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -1303,8 +1324,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G33" s="27"/>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -1313,7 +1335,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -1322,7 +1344,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -1331,43 +1353,43 @@
         <v>-</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="4"/>
-      <c r="C37" s="7"/>
+      <c r="C37" s="4"/>
       <c r="D37" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
-      <c r="B38" s="11"/>
+      <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
+      <c r="C39" s="7"/>
       <c r="D39" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="8"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="4"/>
       <c r="D40" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -1376,16 +1398,16 @@
         <v>-</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
+      <c r="C42" s="8"/>
       <c r="D42" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -1394,7 +1416,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -1403,7 +1425,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -1412,7 +1434,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -1421,7 +1443,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="9"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -1430,7 +1452,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -1439,7 +1461,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -1448,7 +1470,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -1457,7 +1479,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -1466,43 +1488,43 @@
         <v>-</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="9"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="9"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
       <c r="D53" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
+      <c r="B54" s="5"/>
+      <c r="C54" s="9"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="9"/>
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
       <c r="D55" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -1511,7 +1533,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -1520,7 +1542,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -1529,7 +1551,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="9"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -1538,7 +1560,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="9"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -1547,7 +1569,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="9"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -1556,7 +1578,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="9"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -1565,7 +1587,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="9"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -1574,7 +1596,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="9"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -1582,7 +1604,6 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F64" s="4"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="9"/>
@@ -1592,35 +1613,35 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F65" s="4"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="3" t="str">
-        <f t="shared" ref="D66:D101" si="1">IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
-        <v>-</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F66" s="4"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="9"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F67" s="4"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="9"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="F68" s="4"/>
+        <f t="shared" ref="D68:D103" si="1">IF(C68&lt;&gt;"",IF(B68&lt;&gt;"",C68-B68,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="9"/>
@@ -1630,7 +1651,6 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="F69" s="4"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="9"/>
@@ -1640,6 +1660,7 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="F70" s="4"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="9"/>
@@ -1649,6 +1670,7 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="F71" s="4"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="9"/>
@@ -1748,11 +1770,10 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E82" s="12"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
-      <c r="B83" s="12"/>
+      <c r="B83" s="4"/>
       <c r="C83" s="4"/>
       <c r="D83" s="3" t="str">
         <f t="shared" si="1"/>
@@ -1767,10 +1788,11 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="E84" s="12"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
-      <c r="B85" s="4"/>
+      <c r="B85" s="12"/>
       <c r="C85" s="4"/>
       <c r="D85" s="3" t="str">
         <f t="shared" si="1"/>
@@ -1785,7 +1807,6 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E86" s="4"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="9"/>
@@ -1796,7 +1817,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
@@ -1804,6 +1825,7 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="E88" s="4"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
@@ -1814,7 +1836,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="9"/>
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
@@ -1870,8 +1892,8 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="9"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="6"/>
+      <c r="B96" s="4"/>
+      <c r="C96" s="4"/>
       <c r="D96" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
@@ -1888,8 +1910,8 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="9"/>
-      <c r="B98" s="4"/>
-      <c r="C98" s="4"/>
+      <c r="B98" s="6"/>
+      <c r="C98" s="6"/>
       <c r="D98" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
@@ -1903,7 +1925,6 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E99" s="4"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
@@ -1922,14 +1943,25 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="E101" s="4"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="9"/>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="9"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B104" s="4"/>
@@ -1942,12 +1974,10 @@
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
-      <c r="D106" s="3"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
-      <c r="D107" s="3"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B108" s="4"/>
@@ -1967,10 +1997,12 @@
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
+      <c r="D111" s="3"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
+      <c r="D112" s="3"/>
     </row>
     <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113" s="4"/>
@@ -2263,6 +2295,14 @@
     <row r="185" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B185" s="4"/>
       <c r="C185" s="4"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="4"/>
+      <c r="C186" s="4"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="4"/>
+      <c r="C187" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2587,14 +2627,14 @@
         <v>3</v>
       </c>
       <c r="B19" s="4">
-        <v>39607</v>
+        <v>39967</v>
       </c>
       <c r="C19" s="4">
         <v>39864</v>
       </c>
       <c r="D19" s="3">
         <f t="shared" si="0"/>
-        <v>257</v>
+        <v>-103</v>
       </c>
       <c r="G19" s="24"/>
     </row>

</xml_diff>

<commit_message>
paperboy - v4 done up to saturday, 5 frames saved
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DF878D-E661-44C6-ACB2-3F005DFDBEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69198B1-92A2-4D30-A5EF-A650FE454AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49710" yWindow="2070" windowWidth="8025" windowHeight="12285" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49455" yWindow="2070" windowWidth="8280" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="V3" sheetId="11" r:id="rId1"/>
-    <sheet name="V2" sheetId="9" r:id="rId2"/>
-    <sheet name="V1" sheetId="8" r:id="rId3"/>
-    <sheet name="Bulb Check" sheetId="10" r:id="rId4"/>
+    <sheet name="v4" sheetId="12" r:id="rId1"/>
+    <sheet name="V3" sheetId="11" r:id="rId2"/>
+    <sheet name="V2" sheetId="9" r:id="rId3"/>
+    <sheet name="V1" sheetId="8" r:id="rId4"/>
+    <sheet name="Bulb Check" sheetId="10" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="78">
   <si>
     <t>Place</t>
   </si>
@@ -258,6 +259,15 @@
   </si>
   <si>
     <t>rta v3</t>
+  </si>
+  <si>
+    <t>actual ending</t>
+  </si>
+  <si>
+    <t>Uses actual ending</t>
+  </si>
+  <si>
+    <t>rta v4</t>
   </si>
 </sst>
 </file>
@@ -267,12 +277,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -493,22 +510,23 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -518,23 +536,23 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
@@ -855,6 +873,1429 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD1E4B9-F96C-4FBD-81E5-9B315D7F4F9C}">
+  <dimension ref="A1:G185"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.75" customWidth="1"/>
+    <col min="4" max="4" width="6.625" customWidth="1"/>
+    <col min="5" max="5" width="17.625" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3">
+        <f t="shared" ref="D2:D65" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="15">
+        <v>281</v>
+      </c>
+      <c r="C3" s="15">
+        <v>281</v>
+      </c>
+      <c r="D3" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="15">
+        <v>924</v>
+      </c>
+      <c r="C4" s="15">
+        <v>924</v>
+      </c>
+      <c r="D4" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1804</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1804</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="15">
+        <v>6013</v>
+      </c>
+      <c r="C6" s="15">
+        <v>6013</v>
+      </c>
+      <c r="D6" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="15"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="24"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="2">
+        <v>7397</v>
+      </c>
+      <c r="C7" s="2">
+        <v>7397</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="28"/>
+      <c r="F7" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="24"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="19">
+        <v>11611</v>
+      </c>
+      <c r="C8" s="19">
+        <v>11611</v>
+      </c>
+      <c r="D8" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="24"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4">
+        <v>12995</v>
+      </c>
+      <c r="C9" s="4">
+        <v>12995</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="24"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="19">
+        <v>17212</v>
+      </c>
+      <c r="C10" s="19">
+        <v>17212</v>
+      </c>
+      <c r="D10" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E10" s="17"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="24"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="4">
+        <v>18596</v>
+      </c>
+      <c r="C11" s="4">
+        <v>18596</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="24"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="19">
+        <v>22827</v>
+      </c>
+      <c r="C12" s="19">
+        <v>22828</v>
+      </c>
+      <c r="D12" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E12" s="17"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="24"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="4">
+        <v>24211</v>
+      </c>
+      <c r="C13" s="4">
+        <v>24212</v>
+      </c>
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="19">
+        <v>28457</v>
+      </c>
+      <c r="C14" s="19">
+        <v>28462</v>
+      </c>
+      <c r="D14" s="16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G14" s="24"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4">
+        <v>29841</v>
+      </c>
+      <c r="C15" s="4">
+        <v>29846</v>
+      </c>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G15" s="24"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4">
+        <v>39967</v>
+      </c>
+      <c r="D18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="9"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G20" s="24"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G21" s="24"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G23" s="24"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G24" s="24"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G25" s="24"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="9"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="9"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G27" s="24"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="9"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G28" s="24"/>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G29" s="24"/>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G30" s="24"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G31" s="27"/>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="9"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="9"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="9"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="9"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="9"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="9"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="9"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="9"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="9"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="9"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="9"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="9"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="9"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="9"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="9"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="9"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="9"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="9"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="9"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="9"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="9"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="9"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="9"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="9"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="9"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="9"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="9"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="9"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F64" s="4"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="9"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F65" s="4"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="9"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="3" t="str">
+        <f t="shared" ref="D66:D101" si="1">IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="9"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="9"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="F68" s="4"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="9"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="F69" s="4"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="9"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="9"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="9"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="9"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="9"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="9"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="9"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="9"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="9"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="9"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="9"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="9"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="9"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E82" s="12"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="9"/>
+      <c r="B83" s="12"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="9"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="9"/>
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="9"/>
+      <c r="B86" s="4"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E86" s="4"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="9"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="9"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="9"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="9"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="9"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="9"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="9"/>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="9"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="9"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="9"/>
+      <c r="B96" s="6"/>
+      <c r="C96" s="6"/>
+      <c r="D96" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="9"/>
+      <c r="B97" s="4"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="9"/>
+      <c r="B98" s="4"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="9"/>
+      <c r="B99" s="4"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E99" s="4"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="9"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="9"/>
+      <c r="B101" s="4"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B102" s="4"/>
+      <c r="C102" s="4"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B103" s="4"/>
+      <c r="C103" s="4"/>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B105" s="4"/>
+      <c r="C105" s="4"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="3"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B107" s="4"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="3"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B108" s="4"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="3"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B109" s="4"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="3"/>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B110" s="4"/>
+      <c r="C110" s="4"/>
+      <c r="D110" s="3"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B111" s="4"/>
+      <c r="C111" s="4"/>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B112" s="4"/>
+      <c r="C112" s="4"/>
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B113" s="4"/>
+      <c r="C113" s="4"/>
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B114" s="4"/>
+      <c r="C114" s="4"/>
+    </row>
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B115" s="4"/>
+      <c r="C115" s="4"/>
+    </row>
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B116" s="4"/>
+      <c r="C116" s="4"/>
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B117" s="4"/>
+      <c r="C117" s="4"/>
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B118" s="4"/>
+      <c r="C118" s="4"/>
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B119" s="4"/>
+      <c r="C119" s="4"/>
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B120" s="4"/>
+      <c r="C120" s="4"/>
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B121" s="4"/>
+      <c r="C121" s="4"/>
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B122" s="4"/>
+      <c r="C122" s="4"/>
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B123" s="4"/>
+      <c r="C123" s="4"/>
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B124" s="4"/>
+      <c r="C124" s="4"/>
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B125" s="4"/>
+      <c r="C125" s="4"/>
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B126" s="4"/>
+      <c r="C126" s="4"/>
+    </row>
+    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B127" s="4"/>
+      <c r="C127" s="4"/>
+    </row>
+    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B128" s="4"/>
+      <c r="C128" s="4"/>
+    </row>
+    <row r="129" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B129" s="4"/>
+      <c r="C129" s="4"/>
+    </row>
+    <row r="130" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B130" s="4"/>
+      <c r="C130" s="4"/>
+    </row>
+    <row r="131" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B131" s="4"/>
+      <c r="C131" s="4"/>
+    </row>
+    <row r="132" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B132" s="4"/>
+      <c r="C132" s="4"/>
+    </row>
+    <row r="133" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B133" s="4"/>
+      <c r="C133" s="4"/>
+    </row>
+    <row r="134" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B134" s="4"/>
+      <c r="C134" s="4"/>
+    </row>
+    <row r="135" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B135" s="4"/>
+      <c r="C135" s="4"/>
+    </row>
+    <row r="136" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B136" s="4"/>
+      <c r="C136" s="4"/>
+    </row>
+    <row r="137" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B137" s="4"/>
+      <c r="C137" s="4"/>
+    </row>
+    <row r="138" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B138" s="4"/>
+      <c r="C138" s="4"/>
+    </row>
+    <row r="139" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B139" s="4"/>
+      <c r="C139" s="4"/>
+    </row>
+    <row r="140" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B140" s="4"/>
+      <c r="C140" s="4"/>
+    </row>
+    <row r="141" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B141" s="4"/>
+      <c r="C141" s="4"/>
+    </row>
+    <row r="142" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B142" s="4"/>
+      <c r="C142" s="4"/>
+    </row>
+    <row r="143" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B143" s="4"/>
+      <c r="C143" s="4"/>
+    </row>
+    <row r="144" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B144" s="4"/>
+      <c r="C144" s="4"/>
+    </row>
+    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B145" s="4"/>
+      <c r="C145" s="4"/>
+    </row>
+    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B146" s="4"/>
+      <c r="C146" s="4"/>
+    </row>
+    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B147" s="4"/>
+      <c r="C147" s="4"/>
+    </row>
+    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B148" s="4"/>
+      <c r="C148" s="4"/>
+    </row>
+    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B149" s="4"/>
+      <c r="C149" s="4"/>
+    </row>
+    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B150" s="4"/>
+      <c r="C150" s="4"/>
+    </row>
+    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B151" s="4"/>
+      <c r="C151" s="4"/>
+    </row>
+    <row r="152" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B152" s="4"/>
+      <c r="C152" s="4"/>
+    </row>
+    <row r="153" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B153" s="4"/>
+      <c r="C153" s="4"/>
+    </row>
+    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B154" s="4"/>
+      <c r="C154" s="4"/>
+    </row>
+    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B155" s="4"/>
+      <c r="C155" s="4"/>
+    </row>
+    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B156" s="4"/>
+      <c r="C156" s="4"/>
+    </row>
+    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B157" s="4"/>
+      <c r="C157" s="4"/>
+    </row>
+    <row r="158" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B158" s="4"/>
+      <c r="C158" s="4"/>
+    </row>
+    <row r="159" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B159" s="4"/>
+      <c r="C159" s="4"/>
+    </row>
+    <row r="160" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B160" s="4"/>
+      <c r="C160" s="4"/>
+    </row>
+    <row r="161" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B161" s="4"/>
+      <c r="C161" s="4"/>
+    </row>
+    <row r="162" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B162" s="4"/>
+      <c r="C162" s="4"/>
+    </row>
+    <row r="163" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B163" s="4"/>
+      <c r="C163" s="4"/>
+    </row>
+    <row r="164" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B164" s="4"/>
+      <c r="C164" s="4"/>
+    </row>
+    <row r="165" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B165" s="4"/>
+      <c r="C165" s="4"/>
+    </row>
+    <row r="166" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B166" s="4"/>
+      <c r="C166" s="4"/>
+    </row>
+    <row r="167" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B167" s="4"/>
+      <c r="C167" s="4"/>
+    </row>
+    <row r="168" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B168" s="4"/>
+      <c r="C168" s="4"/>
+    </row>
+    <row r="169" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B169" s="4"/>
+      <c r="C169" s="4"/>
+    </row>
+    <row r="170" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B170" s="4"/>
+      <c r="C170" s="4"/>
+    </row>
+    <row r="171" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B171" s="4"/>
+      <c r="C171" s="4"/>
+    </row>
+    <row r="172" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B172" s="4"/>
+      <c r="C172" s="4"/>
+    </row>
+    <row r="173" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B173" s="4"/>
+      <c r="C173" s="4"/>
+    </row>
+    <row r="174" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B174" s="4"/>
+      <c r="C174" s="4"/>
+    </row>
+    <row r="175" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B175" s="4"/>
+      <c r="C175" s="4"/>
+    </row>
+    <row r="176" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B176" s="4"/>
+      <c r="C176" s="4"/>
+    </row>
+    <row r="177" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B177" s="4"/>
+      <c r="C177" s="4"/>
+    </row>
+    <row r="178" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B178" s="4"/>
+      <c r="C178" s="4"/>
+    </row>
+    <row r="179" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B179" s="4"/>
+      <c r="C179" s="4"/>
+    </row>
+    <row r="180" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B180" s="4"/>
+      <c r="C180" s="4"/>
+    </row>
+    <row r="181" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B181" s="4"/>
+      <c r="C181" s="4"/>
+    </row>
+    <row r="182" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B182" s="4"/>
+      <c r="C182" s="4"/>
+    </row>
+    <row r="183" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B183" s="4"/>
+      <c r="C183" s="4"/>
+    </row>
+    <row r="184" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B184" s="4"/>
+      <c r="C184" s="4"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="4"/>
+      <c r="C185" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FBDE017-57E1-41A6-9366-1949A55961DE}">
   <dimension ref="A1:G187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1185,14 +2626,17 @@
         <v>3</v>
       </c>
       <c r="B20" s="4">
-        <v>39524</v>
+        <v>39967</v>
       </c>
       <c r="C20" s="4">
         <v>39607</v>
       </c>
       <c r="D20" s="3">
         <f t="shared" si="0"/>
-        <v>83</v>
+        <v>-360</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>76</v>
       </c>
       <c r="G20" s="24"/>
     </row>
@@ -2310,7 +3754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1983864C-ED7D-4E0B-969E-AE843FEB855D}">
   <dimension ref="A1:G186"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2626,15 +4070,16 @@
       <c r="A19" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="4">
-        <v>39967</v>
-      </c>
+      <c r="B19" s="4"/>
       <c r="C19" s="4">
         <v>39864</v>
       </c>
-      <c r="D19" s="3">
-        <f t="shared" si="0"/>
-        <v>-103</v>
+      <c r="D19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>75</v>
       </c>
       <c r="G19" s="24"/>
     </row>
@@ -3752,7 +5197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
   <dimension ref="A1:I185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5249,7 +6694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAC1BD0-BE10-4CBC-A8BB-B931744D8671}">
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
paperboy - rta v4 done, 16 frames faster than v3
</commit_message>
<xml_diff>
--- a/Paperboy/compare.xlsx
+++ b/Paperboy/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\Paperboy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69198B1-92A2-4D30-A5EF-A650FE454AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FACB297-66B8-418E-ACC4-761F7A3EBF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49455" yWindow="2070" windowWidth="8280" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="91">
   <si>
     <t>Place</t>
   </si>
@@ -268,6 +268,45 @@
   </si>
   <si>
     <t>rta v4</t>
+  </si>
+  <si>
+    <t>end house 3</t>
+  </si>
+  <si>
+    <t>to dog 1</t>
+  </si>
+  <si>
+    <t>after tricyclist</t>
+  </si>
+  <si>
+    <t>Hit 1st dog with paper</t>
+  </si>
+  <si>
+    <t>Newspaper pickup white house</t>
+  </si>
+  <si>
+    <t>end white house</t>
+  </si>
+  <si>
+    <t>Grim reaper</t>
+  </si>
+  <si>
+    <t>before skateboarder</t>
+  </si>
+  <si>
+    <t>last papers on block</t>
+  </si>
+  <si>
+    <t>Block 2</t>
+  </si>
+  <si>
+    <t>pkg 2nd house</t>
+  </si>
+  <si>
+    <t>2 pkgs later</t>
+  </si>
+  <si>
+    <t>pkg</t>
   </si>
 </sst>
 </file>
@@ -277,12 +316,26 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -510,22 +563,24 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -534,26 +589,27 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -874,7 +930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD1E4B9-F96C-4FBD-81E5-9B315D7F4F9C}">
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G202"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
@@ -910,7 +966,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D65" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D82" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>0</v>
       </c>
     </row>
@@ -1141,213 +1197,325 @@
       <c r="G15" s="24"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="4">
+        <v>7949</v>
+      </c>
+      <c r="C16" s="4">
+        <v>7954</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="4">
+        <v>7952</v>
+      </c>
+      <c r="C17" s="4">
+        <v>7957</v>
+      </c>
+      <c r="D17" s="3">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="4">
+        <v>7978</v>
+      </c>
+      <c r="C18" s="4">
+        <v>7984</v>
+      </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4">
+        <v>7981</v>
+      </c>
+      <c r="C19" s="4">
+        <v>7987</v>
+      </c>
+      <c r="D19" s="3">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="4">
+        <v>8024</v>
+      </c>
+      <c r="C20" s="4">
+        <v>8030</v>
+      </c>
+      <c r="D20" s="3">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="G20" s="24"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G16" s="24"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+      <c r="B21" s="29">
+        <v>34181</v>
+      </c>
+      <c r="C21" s="29">
+        <v>34191</v>
+      </c>
+      <c r="D21" s="16">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G21" s="24"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G17" s="24"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="B22" s="4">
+        <v>35565</v>
+      </c>
+      <c r="C22" s="4">
+        <v>35575</v>
+      </c>
+      <c r="D22" s="3">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="4">
+        <v>9482</v>
+      </c>
+      <c r="C23" s="4">
+        <v>9493</v>
+      </c>
+      <c r="D23" s="16">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G23" s="24"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" s="4">
+        <v>9499</v>
+      </c>
+      <c r="C24" s="4">
+        <v>9510</v>
+      </c>
+      <c r="D24" s="34">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G24" s="24"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="4">
+        <v>9505</v>
+      </c>
+      <c r="C25" s="4">
+        <v>9516</v>
+      </c>
+      <c r="D25" s="34">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G25" s="24"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="4">
+        <v>9516</v>
+      </c>
+      <c r="C26" s="4">
+        <v>9527</v>
+      </c>
+      <c r="D26" s="34">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="4">
+        <v>9537</v>
+      </c>
+      <c r="C27" s="4">
+        <v>9548</v>
+      </c>
+      <c r="D27" s="34">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G27" s="24"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="4">
+        <v>9564</v>
+      </c>
+      <c r="C28" s="4">
+        <v>9577</v>
+      </c>
+      <c r="D28" s="34">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G28" s="24"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="B29" s="4">
+        <v>9567</v>
+      </c>
+      <c r="C29" s="4">
+        <v>9580</v>
+      </c>
+      <c r="D29" s="34">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G29" s="24"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="4">
+        <v>9569</v>
+      </c>
+      <c r="C30" s="4">
+        <v>9582</v>
+      </c>
+      <c r="D30" s="34">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G30" s="24"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" s="4">
+        <v>9576</v>
+      </c>
+      <c r="C31" s="4">
+        <v>9589</v>
+      </c>
+      <c r="D31" s="34">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G31" s="24"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="4">
+        <v>9583</v>
+      </c>
+      <c r="C32" s="4">
+        <v>9597</v>
+      </c>
+      <c r="D32" s="34">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="G32" s="24"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="33"/>
+      <c r="B33" s="4">
+        <v>9584</v>
+      </c>
+      <c r="C33" s="4">
+        <v>9598</v>
+      </c>
+      <c r="D33" s="34">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="G33" s="24"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="33"/>
+      <c r="B34" s="4">
+        <v>9639</v>
+      </c>
+      <c r="C34" s="4">
+        <v>9655</v>
+      </c>
+      <c r="D34" s="34">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="G34" s="24"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4">
+      <c r="B35" s="4">
+        <v>39951</v>
+      </c>
+      <c r="C35" s="4">
         <v>39967</v>
       </c>
-      <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E18" s="31" t="s">
+      <c r="D35" s="3">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="E35" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="24"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G19" s="24"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G20" s="24"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G21" s="24"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G22" s="24"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G23" s="24"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="9"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G24" s="24"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G25" s="24"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="9"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G26" s="24"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G27" s="24"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="9"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G28" s="24"/>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G29" s="24"/>
-    </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G30" s="24"/>
-    </row>
-    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="G31" s="27"/>
-    </row>
-    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="9"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G35" s="24"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -1355,26 +1523,29 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G36" s="24"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="4"/>
-      <c r="C37" s="7"/>
+      <c r="C37" s="4"/>
       <c r="D37" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G37" s="24"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
-      <c r="B38" s="11"/>
+      <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G38" s="24"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -1382,17 +1553,19 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G39" s="24"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
       <c r="B40" s="4"/>
-      <c r="C40" s="8"/>
+      <c r="C40" s="4"/>
       <c r="D40" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G40" s="24"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -1400,8 +1573,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G41" s="24"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -1409,8 +1583,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G42" s="24"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -1418,8 +1593,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G43" s="24"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -1427,17 +1603,19 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G44" s="24"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
-      <c r="B45" s="4"/>
+      <c r="B45" s="10"/>
       <c r="C45" s="4"/>
       <c r="D45" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G45" s="24"/>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -1445,8 +1623,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G46" s="24"/>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -1454,8 +1633,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G47" s="24"/>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -1463,8 +1643,9 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" s="27"/>
+    </row>
+    <row r="49" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -1473,7 +1654,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -1482,7 +1663,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -1491,43 +1672,43 @@
         <v>-</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="9"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="9"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
       <c r="D53" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
       <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
+      <c r="C54" s="7"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="9"/>
-      <c r="B55" s="4"/>
+      <c r="B55" s="11"/>
       <c r="C55" s="4"/>
       <c r="D55" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -1536,16 +1717,16 @@
         <v>-</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
       <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
+      <c r="C57" s="8"/>
       <c r="D57" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -1554,7 +1735,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="9"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -1563,7 +1744,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="9"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -1572,7 +1753,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="9"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -1581,7 +1762,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="9"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -1590,7 +1771,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="9"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -1599,7 +1780,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="9"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -1607,9 +1788,8 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F64" s="4"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="9"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -1617,174 +1797,172 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F65" s="4"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="3" t="str">
-        <f t="shared" ref="D66:D101" si="1">IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="9"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="9"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="F68" s="4"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="9"/>
-      <c r="B69" s="4"/>
-      <c r="C69" s="4"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="9"/>
       <c r="D69" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="F69" s="4"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="9"/>
-      <c r="B70" s="4"/>
-      <c r="C70" s="4"/>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
       <c r="D70" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="9"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="9"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
       <c r="D72" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="9"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
       <c r="D73" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="9"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
       <c r="D74" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="9"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
       <c r="D75" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="9"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
       <c r="D76" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="9"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
       <c r="D77" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="9"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
       <c r="D78" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="9"/>
       <c r="B79" s="4"/>
       <c r="C79" s="4"/>
       <c r="D79" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="9"/>
       <c r="B80" s="4"/>
       <c r="C80" s="4"/>
       <c r="D80" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="9"/>
       <c r="B81" s="4"/>
       <c r="C81" s="4"/>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F81" s="4"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="9"/>
       <c r="B82" s="4"/>
       <c r="C82" s="4"/>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E82" s="12"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="F82" s="4"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
-      <c r="B83" s="12"/>
+      <c r="B83" s="4"/>
       <c r="C83" s="4"/>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D83:D118" si="1">IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="9"/>
       <c r="B84" s="4"/>
       <c r="C84" s="4"/>
@@ -1793,7 +1971,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
@@ -1801,8 +1979,9 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F85" s="4"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
@@ -1810,9 +1989,9 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E86" s="4"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F86" s="4"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="9"/>
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
@@ -1821,7 +2000,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
@@ -1830,7 +2009,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
@@ -1839,7 +2018,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="9"/>
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
@@ -1848,7 +2027,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="9"/>
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
@@ -1857,7 +2036,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
@@ -1866,7 +2045,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="9"/>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
@@ -1875,7 +2054,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="9"/>
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
@@ -1884,7 +2063,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
@@ -1893,10 +2072,10 @@
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="9"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="6"/>
+      <c r="B96" s="4"/>
+      <c r="C96" s="4"/>
       <c r="D96" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
@@ -1928,11 +2107,11 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E99" s="4"/>
+      <c r="E99" s="12"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
-      <c r="B100" s="4"/>
+      <c r="B100" s="12"/>
       <c r="C100" s="4"/>
       <c r="D100" s="3" t="str">
         <f t="shared" si="1"/>
@@ -1949,115 +2128,202 @@
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="9"/>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="9"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E103" s="4"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="9"/>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="9"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="9"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
-      <c r="D106" s="3"/>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="9"/>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
-      <c r="D107" s="3"/>
+      <c r="D107" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="9"/>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
-      <c r="D108" s="3"/>
+      <c r="D108" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="9"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
-      <c r="D109" s="3"/>
+      <c r="D109" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="9"/>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
-      <c r="D110" s="3"/>
+      <c r="D110" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="9"/>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
+      <c r="D111" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="9"/>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B113" s="4"/>
-      <c r="C113" s="4"/>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D112" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="9"/>
+      <c r="B113" s="6"/>
+      <c r="C113" s="6"/>
+      <c r="D113" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="9"/>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
-    </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D114" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="9"/>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
-    </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D115" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="9"/>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
-    </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D116" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E116" s="4"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="9"/>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
-    </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D117" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="9"/>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
-    </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D118" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
-    </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D123" s="3"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
-    </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D124" s="3"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
-    </row>
-    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D125" s="3"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B126" s="4"/>
       <c r="C126" s="4"/>
-    </row>
-    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D126" s="3"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B127" s="4"/>
       <c r="C127" s="4"/>
-    </row>
-    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D127" s="3"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B128" s="4"/>
       <c r="C128" s="4"/>
     </row>
@@ -2288,6 +2554,74 @@
     <row r="185" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B185" s="4"/>
       <c r="C185" s="4"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="4"/>
+      <c r="C186" s="4"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="4"/>
+      <c r="C187" s="4"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="4"/>
+      <c r="C188" s="4"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="4"/>
+      <c r="C189" s="4"/>
+    </row>
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B190" s="4"/>
+      <c r="C190" s="4"/>
+    </row>
+    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B191" s="4"/>
+      <c r="C191" s="4"/>
+    </row>
+    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B192" s="4"/>
+      <c r="C192" s="4"/>
+    </row>
+    <row r="193" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B193" s="4"/>
+      <c r="C193" s="4"/>
+    </row>
+    <row r="194" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B194" s="4"/>
+      <c r="C194" s="4"/>
+    </row>
+    <row r="195" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B195" s="4"/>
+      <c r="C195" s="4"/>
+    </row>
+    <row r="196" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B196" s="4"/>
+      <c r="C196" s="4"/>
+    </row>
+    <row r="197" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B197" s="4"/>
+      <c r="C197" s="4"/>
+    </row>
+    <row r="198" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B198" s="4"/>
+      <c r="C198" s="4"/>
+    </row>
+    <row r="199" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B199" s="4"/>
+      <c r="C199" s="4"/>
+    </row>
+    <row r="200" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B200" s="4"/>
+      <c r="C200" s="4"/>
+    </row>
+    <row r="201" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B201" s="4"/>
+      <c r="C201" s="4"/>
+    </row>
+    <row r="202" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B202" s="4"/>
+      <c r="C202" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>